<commit_message>
Done #181, plus completed some tests along the way
</commit_message>
<xml_diff>
--- a/tests/data/post_clearcut_allom.xlsx
+++ b/tests/data/post_clearcut_allom.xlsx
@@ -417,30 +417,7 @@
   <dimension ref="A1:V21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr"/>
-      <c r="B1" t="inlineStr"/>
-      <c r="C1" t="inlineStr"/>
-      <c r="D1" t="inlineStr"/>
-      <c r="E1" t="inlineStr"/>
-      <c r="F1" t="inlineStr"/>
-      <c r="G1" t="inlineStr"/>
-      <c r="H1" t="inlineStr"/>
-      <c r="I1" t="inlineStr"/>
-      <c r="J1" t="inlineStr"/>
-      <c r="K1" t="inlineStr"/>
-      <c r="L1" t="inlineStr"/>
-      <c r="M1" t="inlineStr"/>
-      <c r="N1" t="inlineStr"/>
-      <c r="O1" t="inlineStr"/>
-      <c r="P1" t="inlineStr"/>
-      <c r="Q1" t="inlineStr"/>
-      <c r="R1" t="inlineStr"/>
-      <c r="S1" t="inlineStr"/>
-      <c r="T1" t="inlineStr"/>
-      <c r="U1" t="inlineStr"/>
-      <c r="V1" t="inlineStr"/>
-    </row>
+    <row r="1"/>
     <row r="2">
       <c r="A2" t="n">
         <v>1</v>
@@ -452,61 +429,61 @@
         <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>1000</v>
+        <v>5937.5</v>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>0.649</v>
       </c>
       <c r="F2" t="n">
-        <v>0.1</v>
+        <v>0.19</v>
       </c>
       <c r="G2" t="n">
-        <v>1</v>
+        <v>0.26</v>
       </c>
       <c r="H2" t="n">
-        <v>10</v>
+        <v>0.21</v>
       </c>
       <c r="I2" t="n">
-        <v>1</v>
+        <v>0.79</v>
       </c>
       <c r="J2" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>0.1</v>
+        <v>0.24</v>
       </c>
       <c r="L2" t="n">
-        <v>0.1</v>
+        <v>0.016</v>
       </c>
       <c r="M2" t="n">
-        <v>0.5</v>
+        <v>0.83</v>
       </c>
       <c r="N2" t="n">
-        <v>0</v>
+        <v>0.018</v>
       </c>
       <c r="O2" t="n">
-        <v>0</v>
+        <v>0.627</v>
       </c>
       <c r="P2" t="n">
-        <v>0.1</v>
+        <v>0.0125</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.05</v>
+        <v>0.0502</v>
       </c>
       <c r="R2" t="n">
-        <v>0.5</v>
+        <v>0.0002</v>
       </c>
       <c r="S2" t="n">
-        <v>0.1</v>
+        <v>2.031</v>
       </c>
       <c r="T2" t="n">
-        <v>0.1</v>
+        <v>0.06270000000000001</v>
       </c>
       <c r="U2" t="n">
-        <v>0.5</v>
+        <v>0.094</v>
       </c>
       <c r="V2" t="n">
-        <v>0.05</v>
+        <v>0.0325</v>
       </c>
     </row>
     <row r="3">
@@ -520,61 +497,61 @@
         <v>6</v>
       </c>
       <c r="D3" t="n">
-        <v>1000</v>
+        <v>5625</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>2.72</v>
       </c>
       <c r="F3" t="n">
-        <v>0.1</v>
+        <v>1.12</v>
       </c>
       <c r="G3" t="n">
-        <v>1</v>
+        <v>1.56</v>
       </c>
       <c r="H3" t="n">
-        <v>10</v>
+        <v>1.25</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>8.16</v>
       </c>
       <c r="J3" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>0.1</v>
+        <v>2.45</v>
       </c>
       <c r="L3" t="n">
-        <v>0.1</v>
+        <v>0.163</v>
       </c>
       <c r="M3" t="n">
-        <v>0.5</v>
+        <v>8.57</v>
       </c>
       <c r="N3" t="n">
-        <v>0</v>
+        <v>0.092</v>
       </c>
       <c r="O3" t="n">
-        <v>0</v>
+        <v>5.385</v>
       </c>
       <c r="P3" t="n">
-        <v>0.1</v>
+        <v>0.1077</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.05</v>
+        <v>0.4308</v>
       </c>
       <c r="R3" t="n">
-        <v>0.5</v>
+        <v>0.0101</v>
       </c>
       <c r="S3" t="n">
-        <v>0.1</v>
+        <v>2.188</v>
       </c>
       <c r="T3" t="n">
-        <v>0.1</v>
+        <v>0.5385</v>
       </c>
       <c r="U3" t="n">
-        <v>0.5</v>
+        <v>0.8077</v>
       </c>
       <c r="V3" t="n">
-        <v>0.05</v>
+        <v>0.1277</v>
       </c>
     </row>
     <row r="4">
@@ -588,61 +565,61 @@
         <v>11</v>
       </c>
       <c r="D4" t="n">
-        <v>1000</v>
+        <v>5312.5</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>4.418</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1</v>
+        <v>2.06</v>
       </c>
       <c r="G4" t="n">
-        <v>1</v>
+        <v>2.86</v>
       </c>
       <c r="H4" t="n">
-        <v>10</v>
+        <v>2.29</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>17.95</v>
       </c>
       <c r="J4" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>0.1</v>
+        <v>5.38</v>
       </c>
       <c r="L4" t="n">
-        <v>0.1</v>
+        <v>0.359</v>
       </c>
       <c r="M4" t="n">
-        <v>0.5</v>
+        <v>18.85</v>
       </c>
       <c r="N4" t="n">
-        <v>0</v>
+        <v>0.19</v>
       </c>
       <c r="O4" t="n">
-        <v>0</v>
+        <v>11.144</v>
       </c>
       <c r="P4" t="n">
-        <v>0.1</v>
+        <v>0.2229</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.05</v>
+        <v>0.8915</v>
       </c>
       <c r="R4" t="n">
-        <v>0.5</v>
+        <v>0.0383</v>
       </c>
       <c r="S4" t="n">
-        <v>0.1</v>
+        <v>2.344</v>
       </c>
       <c r="T4" t="n">
-        <v>0.1</v>
+        <v>1.1144</v>
       </c>
       <c r="U4" t="n">
-        <v>0.5</v>
+        <v>1.6716</v>
       </c>
       <c r="V4" t="n">
-        <v>0.05</v>
+        <v>0.2429</v>
       </c>
     </row>
     <row r="5">
@@ -656,61 +633,61 @@
         <v>16</v>
       </c>
       <c r="D5" t="n">
-        <v>1000</v>
+        <v>5000</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>5.962</v>
       </c>
       <c r="F5" t="n">
-        <v>0.1</v>
+        <v>3</v>
       </c>
       <c r="G5" t="n">
-        <v>1</v>
+        <v>4.17</v>
       </c>
       <c r="H5" t="n">
-        <v>10</v>
+        <v>3.33</v>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>29.21</v>
       </c>
       <c r="J5" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>0.1</v>
+        <v>8.76</v>
       </c>
       <c r="L5" t="n">
-        <v>0.1</v>
+        <v>0.584</v>
       </c>
       <c r="M5" t="n">
-        <v>0.5</v>
+        <v>30.67</v>
       </c>
       <c r="N5" t="n">
-        <v>0</v>
+        <v>0.302</v>
       </c>
       <c r="O5" t="n">
-        <v>0</v>
+        <v>17.471</v>
       </c>
       <c r="P5" t="n">
-        <v>0.1</v>
+        <v>0.3494</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.05</v>
+        <v>1.3977</v>
       </c>
       <c r="R5" t="n">
-        <v>0.5</v>
+        <v>0.08740000000000001</v>
       </c>
       <c r="S5" t="n">
-        <v>0.1</v>
+        <v>2.5</v>
       </c>
       <c r="T5" t="n">
-        <v>0.1</v>
+        <v>1.7471</v>
       </c>
       <c r="U5" t="n">
-        <v>0.5</v>
+        <v>2.6206</v>
       </c>
       <c r="V5" t="n">
-        <v>0.05</v>
+        <v>0.3694</v>
       </c>
     </row>
     <row r="6">
@@ -724,61 +701,61 @@
         <v>21</v>
       </c>
       <c r="D6" t="n">
-        <v>1000</v>
+        <v>4687.5</v>
       </c>
       <c r="E6" t="n">
-        <v>1</v>
+        <v>7.411</v>
       </c>
       <c r="F6" t="n">
-        <v>0.1</v>
+        <v>3.94</v>
       </c>
       <c r="G6" t="n">
-        <v>1</v>
+        <v>5.47</v>
       </c>
       <c r="H6" t="n">
-        <v>10</v>
+        <v>4.38</v>
       </c>
       <c r="I6" t="n">
-        <v>1</v>
+        <v>41.6</v>
       </c>
       <c r="J6" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>0.1</v>
+        <v>12.48</v>
       </c>
       <c r="L6" t="n">
-        <v>0.1</v>
+        <v>0.832</v>
       </c>
       <c r="M6" t="n">
-        <v>0.5</v>
+        <v>43.68</v>
       </c>
       <c r="N6" t="n">
-        <v>0</v>
+        <v>0.426</v>
       </c>
       <c r="O6" t="n">
-        <v>0</v>
+        <v>24.212</v>
       </c>
       <c r="P6" t="n">
-        <v>0.1</v>
+        <v>0.4842</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.05</v>
+        <v>1.937</v>
       </c>
       <c r="R6" t="n">
-        <v>0.5</v>
+        <v>0.1589</v>
       </c>
       <c r="S6" t="n">
-        <v>0.1</v>
+        <v>2.656</v>
       </c>
       <c r="T6" t="n">
-        <v>0.1</v>
+        <v>2.4212</v>
       </c>
       <c r="U6" t="n">
-        <v>0.5</v>
+        <v>3.6318</v>
       </c>
       <c r="V6" t="n">
-        <v>0.05</v>
+        <v>0.5042</v>
       </c>
     </row>
     <row r="7">
@@ -792,61 +769,61 @@
         <v>26</v>
       </c>
       <c r="D7" t="n">
-        <v>1000</v>
+        <v>4375</v>
       </c>
       <c r="E7" t="n">
-        <v>1</v>
+        <v>8.792</v>
       </c>
       <c r="F7" t="n">
-        <v>0.1</v>
+        <v>4.88</v>
       </c>
       <c r="G7" t="n">
-        <v>1</v>
+        <v>6.77</v>
       </c>
       <c r="H7" t="n">
-        <v>10</v>
+        <v>5.42</v>
       </c>
       <c r="I7" t="n">
-        <v>1</v>
+        <v>54.91</v>
       </c>
       <c r="J7" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>0.1</v>
+        <v>16.47</v>
       </c>
       <c r="L7" t="n">
-        <v>0.1</v>
+        <v>1.098</v>
       </c>
       <c r="M7" t="n">
-        <v>0.5</v>
+        <v>57.66</v>
       </c>
       <c r="N7" t="n">
-        <v>0</v>
+        <v>0.5590000000000001</v>
       </c>
       <c r="O7" t="n">
-        <v>0</v>
+        <v>31.285</v>
       </c>
       <c r="P7" t="n">
-        <v>0.1</v>
+        <v>0.6257</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.05</v>
+        <v>2.5028</v>
       </c>
       <c r="R7" t="n">
-        <v>0.5</v>
+        <v>0.2542</v>
       </c>
       <c r="S7" t="n">
-        <v>0.1</v>
+        <v>2.812</v>
       </c>
       <c r="T7" t="n">
-        <v>0.1</v>
+        <v>3.1285</v>
       </c>
       <c r="U7" t="n">
-        <v>0.5</v>
+        <v>4.6928</v>
       </c>
       <c r="V7" t="n">
-        <v>0.05</v>
+        <v>0.6457000000000001</v>
       </c>
     </row>
     <row r="8">
@@ -860,61 +837,61 @@
         <v>31</v>
       </c>
       <c r="D8" t="n">
-        <v>1000</v>
+        <v>4062.5</v>
       </c>
       <c r="E8" t="n">
-        <v>1</v>
+        <v>10.121</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1</v>
+        <v>5.81</v>
       </c>
       <c r="G8" t="n">
-        <v>1</v>
+        <v>8.07</v>
       </c>
       <c r="H8" t="n">
-        <v>10</v>
+        <v>6.46</v>
       </c>
       <c r="I8" t="n">
-        <v>1</v>
+        <v>69.01000000000001</v>
       </c>
       <c r="J8" t="n">
-        <v>0.5</v>
+        <v>0.99</v>
       </c>
       <c r="K8" t="n">
-        <v>0.1</v>
+        <v>20.7</v>
       </c>
       <c r="L8" t="n">
-        <v>0.1</v>
+        <v>1.38</v>
       </c>
       <c r="M8" t="n">
-        <v>0.5</v>
+        <v>72.45999999999999</v>
       </c>
       <c r="N8" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="O8" t="n">
-        <v>0</v>
+        <v>38.637</v>
       </c>
       <c r="P8" t="n">
-        <v>0.1</v>
+        <v>0.7727000000000001</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.05</v>
+        <v>3.091</v>
       </c>
       <c r="R8" t="n">
-        <v>0.5</v>
+        <v>0.3743</v>
       </c>
       <c r="S8" t="n">
-        <v>0.1</v>
+        <v>2.969</v>
       </c>
       <c r="T8" t="n">
-        <v>0.1</v>
+        <v>3.8637</v>
       </c>
       <c r="U8" t="n">
-        <v>0.5</v>
+        <v>5.7955</v>
       </c>
       <c r="V8" t="n">
-        <v>0.05</v>
+        <v>0.7927</v>
       </c>
     </row>
     <row r="9">
@@ -928,61 +905,61 @@
         <v>36</v>
       </c>
       <c r="D9" t="n">
-        <v>1000</v>
+        <v>3750</v>
       </c>
       <c r="E9" t="n">
-        <v>1</v>
+        <v>11.407</v>
       </c>
       <c r="F9" t="n">
-        <v>0.1</v>
+        <v>6.75</v>
       </c>
       <c r="G9" t="n">
-        <v>1</v>
+        <v>9.380000000000001</v>
       </c>
       <c r="H9" t="n">
-        <v>10</v>
+        <v>7.5</v>
       </c>
       <c r="I9" t="n">
-        <v>1</v>
+        <v>83.81999999999999</v>
       </c>
       <c r="J9" t="n">
-        <v>0.5</v>
+        <v>7.18</v>
       </c>
       <c r="K9" t="n">
-        <v>0.1</v>
+        <v>25.15</v>
       </c>
       <c r="L9" t="n">
-        <v>0.1</v>
+        <v>1.676</v>
       </c>
       <c r="M9" t="n">
-        <v>0.5</v>
+        <v>88.01000000000001</v>
       </c>
       <c r="N9" t="n">
-        <v>0</v>
+        <v>0.848</v>
       </c>
       <c r="O9" t="n">
-        <v>0</v>
+        <v>46.231</v>
       </c>
       <c r="P9" t="n">
-        <v>0.1</v>
+        <v>0.9246</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.05</v>
+        <v>3.6985</v>
       </c>
       <c r="R9" t="n">
-        <v>0.5</v>
+        <v>0.5201</v>
       </c>
       <c r="S9" t="n">
-        <v>0.1</v>
+        <v>3.125</v>
       </c>
       <c r="T9" t="n">
-        <v>0.1</v>
+        <v>4.6231</v>
       </c>
       <c r="U9" t="n">
-        <v>0.5</v>
+        <v>6.9347</v>
       </c>
       <c r="V9" t="n">
-        <v>0.05</v>
+        <v>0.9446</v>
       </c>
     </row>
     <row r="10">
@@ -996,61 +973,61 @@
         <v>41</v>
       </c>
       <c r="D10" t="n">
-        <v>1000</v>
+        <v>3437.5</v>
       </c>
       <c r="E10" t="n">
-        <v>1</v>
+        <v>12.658</v>
       </c>
       <c r="F10" t="n">
-        <v>0.1</v>
+        <v>7.69</v>
       </c>
       <c r="G10" t="n">
-        <v>1</v>
+        <v>10.68</v>
       </c>
       <c r="H10" t="n">
-        <v>10</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="I10" t="n">
-        <v>1</v>
+        <v>99.26000000000001</v>
       </c>
       <c r="J10" t="n">
-        <v>0.5</v>
+        <v>15.6</v>
       </c>
       <c r="K10" t="n">
-        <v>0.1</v>
+        <v>29.78</v>
       </c>
       <c r="L10" t="n">
-        <v>0.1</v>
+        <v>1.985</v>
       </c>
       <c r="M10" t="n">
-        <v>0.5</v>
+        <v>104.22</v>
       </c>
       <c r="N10" t="n">
-        <v>0</v>
+        <v>1.003</v>
       </c>
       <c r="O10" t="n">
-        <v>0</v>
+        <v>54.039</v>
       </c>
       <c r="P10" t="n">
-        <v>0.1</v>
+        <v>1.0808</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.05</v>
+        <v>4.3231</v>
       </c>
       <c r="R10" t="n">
-        <v>0.5</v>
+        <v>0.6924</v>
       </c>
       <c r="S10" t="n">
-        <v>0.1</v>
+        <v>3.281</v>
       </c>
       <c r="T10" t="n">
-        <v>0.1</v>
+        <v>5.4039</v>
       </c>
       <c r="U10" t="n">
-        <v>0.5</v>
+        <v>8.1059</v>
       </c>
       <c r="V10" t="n">
-        <v>0.05</v>
+        <v>1.1008</v>
       </c>
     </row>
     <row r="11">
@@ -1064,61 +1041,61 @@
         <v>46</v>
       </c>
       <c r="D11" t="n">
-        <v>1000</v>
+        <v>3125</v>
       </c>
       <c r="E11" t="n">
-        <v>1</v>
+        <v>13.878</v>
       </c>
       <c r="F11" t="n">
-        <v>0.1</v>
+        <v>8.619999999999999</v>
       </c>
       <c r="G11" t="n">
-        <v>1</v>
+        <v>11.98</v>
       </c>
       <c r="H11" t="n">
-        <v>10</v>
+        <v>9.58</v>
       </c>
       <c r="I11" t="n">
-        <v>1</v>
+        <v>115.28</v>
       </c>
       <c r="J11" t="n">
-        <v>0.5</v>
+        <v>26.35</v>
       </c>
       <c r="K11" t="n">
-        <v>0.1</v>
+        <v>34.58</v>
       </c>
       <c r="L11" t="n">
-        <v>0.1</v>
+        <v>2.306</v>
       </c>
       <c r="M11" t="n">
-        <v>0.5</v>
+        <v>121.04</v>
       </c>
       <c r="N11" t="n">
-        <v>0</v>
+        <v>1.163</v>
       </c>
       <c r="O11" t="n">
-        <v>0</v>
+        <v>62.04</v>
       </c>
       <c r="P11" t="n">
-        <v>0.1</v>
+        <v>1.2408</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.05</v>
+        <v>4.9632</v>
       </c>
       <c r="R11" t="n">
-        <v>0.5</v>
+        <v>0.8918</v>
       </c>
       <c r="S11" t="n">
-        <v>0.1</v>
+        <v>3.438</v>
       </c>
       <c r="T11" t="n">
-        <v>0.1</v>
+        <v>6.204</v>
       </c>
       <c r="U11" t="n">
-        <v>0.5</v>
+        <v>9.305999999999999</v>
       </c>
       <c r="V11" t="n">
-        <v>0.05</v>
+        <v>1.2608</v>
       </c>
     </row>
     <row r="12">
@@ -1132,61 +1109,61 @@
         <v>51</v>
       </c>
       <c r="D12" t="n">
-        <v>1000</v>
+        <v>2812.5</v>
       </c>
       <c r="E12" t="n">
-        <v>1</v>
+        <v>15.072</v>
       </c>
       <c r="F12" t="n">
-        <v>0.1</v>
+        <v>9.56</v>
       </c>
       <c r="G12" t="n">
-        <v>1</v>
+        <v>13.28</v>
       </c>
       <c r="H12" t="n">
-        <v>10</v>
+        <v>10.62</v>
       </c>
       <c r="I12" t="n">
-        <v>1</v>
+        <v>131.83</v>
       </c>
       <c r="J12" t="n">
-        <v>0.5</v>
+        <v>39.55</v>
       </c>
       <c r="K12" t="n">
-        <v>0.1</v>
+        <v>39.55</v>
       </c>
       <c r="L12" t="n">
-        <v>0.1</v>
+        <v>2.637</v>
       </c>
       <c r="M12" t="n">
-        <v>0.5</v>
+        <v>138.42</v>
       </c>
       <c r="N12" t="n">
-        <v>0</v>
+        <v>1.328</v>
       </c>
       <c r="O12" t="n">
-        <v>0</v>
+        <v>70.218</v>
       </c>
       <c r="P12" t="n">
-        <v>0.1</v>
+        <v>1.4044</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.05</v>
+        <v>5.6174</v>
       </c>
       <c r="R12" t="n">
-        <v>0.5</v>
+        <v>1.1191</v>
       </c>
       <c r="S12" t="n">
-        <v>0.1</v>
+        <v>3.594</v>
       </c>
       <c r="T12" t="n">
-        <v>0.1</v>
+        <v>7.0218</v>
       </c>
       <c r="U12" t="n">
-        <v>0.5</v>
+        <v>10.5327</v>
       </c>
       <c r="V12" t="n">
-        <v>0.05</v>
+        <v>1.4244</v>
       </c>
     </row>
     <row r="13">
@@ -1200,61 +1177,61 @@
         <v>56</v>
       </c>
       <c r="D13" t="n">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="E13" t="n">
-        <v>1</v>
+        <v>16.243</v>
       </c>
       <c r="F13" t="n">
-        <v>0.1</v>
+        <v>10.5</v>
       </c>
       <c r="G13" t="n">
-        <v>1</v>
+        <v>14.58</v>
       </c>
       <c r="H13" t="n">
-        <v>10</v>
+        <v>11.67</v>
       </c>
       <c r="I13" t="n">
-        <v>1</v>
+        <v>148.87</v>
       </c>
       <c r="J13" t="n">
-        <v>0.5</v>
+        <v>55.29</v>
       </c>
       <c r="K13" t="n">
-        <v>0.1</v>
+        <v>44.66</v>
       </c>
       <c r="L13" t="n">
-        <v>0.1</v>
+        <v>2.977</v>
       </c>
       <c r="M13" t="n">
-        <v>0.5</v>
+        <v>156.31</v>
       </c>
       <c r="N13" t="n">
-        <v>0</v>
+        <v>1.499</v>
       </c>
       <c r="O13" t="n">
-        <v>0</v>
+        <v>78.55800000000001</v>
       </c>
       <c r="P13" t="n">
-        <v>0.1</v>
+        <v>1.5712</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.05</v>
+        <v>6.2846</v>
       </c>
       <c r="R13" t="n">
-        <v>0.5</v>
+        <v>1.3748</v>
       </c>
       <c r="S13" t="n">
-        <v>0.1</v>
+        <v>3.75</v>
       </c>
       <c r="T13" t="n">
-        <v>0.1</v>
+        <v>7.8558</v>
       </c>
       <c r="U13" t="n">
-        <v>0.5</v>
+        <v>11.7837</v>
       </c>
       <c r="V13" t="n">
-        <v>0.05</v>
+        <v>1.5912</v>
       </c>
     </row>
     <row r="14">
@@ -1268,61 +1245,61 @@
         <v>61</v>
       </c>
       <c r="D14" t="n">
-        <v>1000</v>
+        <v>2187.5</v>
       </c>
       <c r="E14" t="n">
-        <v>1</v>
+        <v>17.393</v>
       </c>
       <c r="F14" t="n">
-        <v>0.1</v>
+        <v>11.44</v>
       </c>
       <c r="G14" t="n">
-        <v>1</v>
+        <v>15.89</v>
       </c>
       <c r="H14" t="n">
-        <v>10</v>
+        <v>12.71</v>
       </c>
       <c r="I14" t="n">
-        <v>1</v>
+        <v>166.38</v>
       </c>
       <c r="J14" t="n">
-        <v>0.5</v>
+        <v>73.68000000000001</v>
       </c>
       <c r="K14" t="n">
-        <v>0.1</v>
+        <v>49.91</v>
       </c>
       <c r="L14" t="n">
-        <v>0.1</v>
+        <v>3.328</v>
       </c>
       <c r="M14" t="n">
-        <v>0.5</v>
+        <v>174.7</v>
       </c>
       <c r="N14" t="n">
-        <v>0</v>
+        <v>1.674</v>
       </c>
       <c r="O14" t="n">
-        <v>0</v>
+        <v>87.04900000000001</v>
       </c>
       <c r="P14" t="n">
-        <v>0.1</v>
+        <v>1.741</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.05</v>
+        <v>6.9639</v>
       </c>
       <c r="R14" t="n">
-        <v>0.5</v>
+        <v>1.6594</v>
       </c>
       <c r="S14" t="n">
-        <v>0.1</v>
+        <v>3.906</v>
       </c>
       <c r="T14" t="n">
-        <v>0.1</v>
+        <v>8.7049</v>
       </c>
       <c r="U14" t="n">
-        <v>0.5</v>
+        <v>13.0574</v>
       </c>
       <c r="V14" t="n">
-        <v>0.05</v>
+        <v>1.761</v>
       </c>
     </row>
     <row r="15">
@@ -1336,61 +1313,61 @@
         <v>66</v>
       </c>
       <c r="D15" t="n">
-        <v>1000</v>
+        <v>1875</v>
       </c>
       <c r="E15" t="n">
-        <v>1</v>
+        <v>18.525</v>
       </c>
       <c r="F15" t="n">
-        <v>0.1</v>
+        <v>12.38</v>
       </c>
       <c r="G15" t="n">
-        <v>1</v>
+        <v>17.19</v>
       </c>
       <c r="H15" t="n">
-        <v>10</v>
+        <v>13.75</v>
       </c>
       <c r="I15" t="n">
-        <v>1</v>
+        <v>184.32</v>
       </c>
       <c r="J15" t="n">
-        <v>0.5</v>
+        <v>94.79000000000001</v>
       </c>
       <c r="K15" t="n">
-        <v>0.1</v>
+        <v>55.3</v>
       </c>
       <c r="L15" t="n">
-        <v>0.1</v>
+        <v>3.686</v>
       </c>
       <c r="M15" t="n">
-        <v>0.5</v>
+        <v>193.54</v>
       </c>
       <c r="N15" t="n">
-        <v>0</v>
+        <v>1.853</v>
       </c>
       <c r="O15" t="n">
-        <v>0</v>
+        <v>95.679</v>
       </c>
       <c r="P15" t="n">
-        <v>0.1</v>
+        <v>1.9136</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.05</v>
+        <v>7.6543</v>
       </c>
       <c r="R15" t="n">
-        <v>0.5</v>
+        <v>1.9734</v>
       </c>
       <c r="S15" t="n">
-        <v>0.1</v>
+        <v>4.062</v>
       </c>
       <c r="T15" t="n">
-        <v>0.1</v>
+        <v>9.5679</v>
       </c>
       <c r="U15" t="n">
-        <v>0.5</v>
+        <v>14.3519</v>
       </c>
       <c r="V15" t="n">
-        <v>0.05</v>
+        <v>1.9336</v>
       </c>
     </row>
     <row r="16">
@@ -1404,61 +1381,61 @@
         <v>71</v>
       </c>
       <c r="D16" t="n">
-        <v>1000</v>
+        <v>1562.5</v>
       </c>
       <c r="E16" t="n">
-        <v>1</v>
+        <v>19.639</v>
       </c>
       <c r="F16" t="n">
-        <v>0.1</v>
+        <v>13.31</v>
       </c>
       <c r="G16" t="n">
-        <v>1</v>
+        <v>18.49</v>
       </c>
       <c r="H16" t="n">
-        <v>10</v>
+        <v>14.79</v>
       </c>
       <c r="I16" t="n">
-        <v>1</v>
+        <v>202.68</v>
       </c>
       <c r="J16" t="n">
-        <v>0.5</v>
+        <v>118.71</v>
       </c>
       <c r="K16" t="n">
-        <v>0.1</v>
+        <v>60.8</v>
       </c>
       <c r="L16" t="n">
-        <v>0.1</v>
+        <v>4.054</v>
       </c>
       <c r="M16" t="n">
-        <v>0.5</v>
+        <v>212.81</v>
       </c>
       <c r="N16" t="n">
-        <v>0</v>
+        <v>2.037</v>
       </c>
       <c r="O16" t="n">
-        <v>0</v>
+        <v>104.442</v>
       </c>
       <c r="P16" t="n">
-        <v>0.1</v>
+        <v>2.0888</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.05</v>
+        <v>8.355399999999999</v>
       </c>
       <c r="R16" t="n">
-        <v>0.5</v>
+        <v>2.3173</v>
       </c>
       <c r="S16" t="n">
-        <v>0.1</v>
+        <v>4.219</v>
       </c>
       <c r="T16" t="n">
-        <v>0.1</v>
+        <v>10.4442</v>
       </c>
       <c r="U16" t="n">
-        <v>0.5</v>
+        <v>15.6663</v>
       </c>
       <c r="V16" t="n">
-        <v>0.05</v>
+        <v>2.1088</v>
       </c>
     </row>
     <row r="17">
@@ -1472,61 +1449,61 @@
         <v>76</v>
       </c>
       <c r="D17" t="n">
-        <v>1000</v>
+        <v>1250</v>
       </c>
       <c r="E17" t="n">
-        <v>1</v>
+        <v>20.738</v>
       </c>
       <c r="F17" t="n">
-        <v>0.1</v>
+        <v>14.25</v>
       </c>
       <c r="G17" t="n">
-        <v>1</v>
+        <v>19.79</v>
       </c>
       <c r="H17" t="n">
-        <v>10</v>
+        <v>15.83</v>
       </c>
       <c r="I17" t="n">
-        <v>1</v>
+        <v>221.42</v>
       </c>
       <c r="J17" t="n">
-        <v>0.5</v>
+        <v>145.5</v>
       </c>
       <c r="K17" t="n">
-        <v>0.1</v>
+        <v>66.43000000000001</v>
       </c>
       <c r="L17" t="n">
-        <v>0.1</v>
+        <v>4.428</v>
       </c>
       <c r="M17" t="n">
-        <v>0.5</v>
+        <v>232.49</v>
       </c>
       <c r="N17" t="n">
-        <v>0</v>
+        <v>2.224</v>
       </c>
       <c r="O17" t="n">
-        <v>0</v>
+        <v>113.329</v>
       </c>
       <c r="P17" t="n">
-        <v>0.1</v>
+        <v>2.2666</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.05</v>
+        <v>9.0663</v>
       </c>
       <c r="R17" t="n">
-        <v>0.5</v>
+        <v>2.6916</v>
       </c>
       <c r="S17" t="n">
-        <v>0.1</v>
+        <v>4.375</v>
       </c>
       <c r="T17" t="n">
-        <v>0.1</v>
+        <v>11.3329</v>
       </c>
       <c r="U17" t="n">
-        <v>0.5</v>
+        <v>16.9993</v>
       </c>
       <c r="V17" t="n">
-        <v>0.05</v>
+        <v>2.2866</v>
       </c>
     </row>
     <row r="18">
@@ -1540,61 +1517,61 @@
         <v>81</v>
       </c>
       <c r="D18" t="n">
-        <v>1000</v>
+        <v>937.5</v>
       </c>
       <c r="E18" t="n">
-        <v>1</v>
+        <v>21.823</v>
       </c>
       <c r="F18" t="n">
-        <v>0.1</v>
+        <v>15.19</v>
       </c>
       <c r="G18" t="n">
-        <v>1</v>
+        <v>21.09</v>
       </c>
       <c r="H18" t="n">
-        <v>10</v>
+        <v>16.88</v>
       </c>
       <c r="I18" t="n">
-        <v>1</v>
+        <v>240.55</v>
       </c>
       <c r="J18" t="n">
-        <v>0.5</v>
+        <v>175.26</v>
       </c>
       <c r="K18" t="n">
-        <v>0.1</v>
+        <v>72.17</v>
       </c>
       <c r="L18" t="n">
-        <v>0.1</v>
+        <v>4.811</v>
       </c>
       <c r="M18" t="n">
-        <v>0.5</v>
+        <v>252.58</v>
       </c>
       <c r="N18" t="n">
-        <v>0</v>
+        <v>2.415</v>
       </c>
       <c r="O18" t="n">
-        <v>0</v>
+        <v>122.334</v>
       </c>
       <c r="P18" t="n">
-        <v>0.1</v>
+        <v>2.4467</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.05</v>
+        <v>9.7867</v>
       </c>
       <c r="R18" t="n">
-        <v>0.5</v>
+        <v>3.0966</v>
       </c>
       <c r="S18" t="n">
-        <v>0.1</v>
+        <v>4.531</v>
       </c>
       <c r="T18" t="n">
-        <v>0.1</v>
+        <v>12.2334</v>
       </c>
       <c r="U18" t="n">
-        <v>0.5</v>
+        <v>18.3501</v>
       </c>
       <c r="V18" t="n">
-        <v>0.05</v>
+        <v>2.4667</v>
       </c>
     </row>
     <row r="19">
@@ -1608,61 +1585,61 @@
         <v>86</v>
       </c>
       <c r="D19" t="n">
-        <v>1000</v>
+        <v>625</v>
       </c>
       <c r="E19" t="n">
-        <v>1</v>
+        <v>22.894</v>
       </c>
       <c r="F19" t="n">
-        <v>0.1</v>
+        <v>16.12</v>
       </c>
       <c r="G19" t="n">
-        <v>1</v>
+        <v>22.4</v>
       </c>
       <c r="H19" t="n">
-        <v>10</v>
+        <v>17.92</v>
       </c>
       <c r="I19" t="n">
-        <v>1</v>
+        <v>260.03</v>
       </c>
       <c r="J19" t="n">
-        <v>0.5</v>
+        <v>208.02</v>
       </c>
       <c r="K19" t="n">
-        <v>0.1</v>
+        <v>78.01000000000001</v>
       </c>
       <c r="L19" t="n">
-        <v>0.1</v>
+        <v>5.201</v>
       </c>
       <c r="M19" t="n">
-        <v>0.5</v>
+        <v>273.03</v>
       </c>
       <c r="N19" t="n">
-        <v>0</v>
+        <v>2.61</v>
       </c>
       <c r="O19" t="n">
-        <v>0</v>
+        <v>131.451</v>
       </c>
       <c r="P19" t="n">
-        <v>0.1</v>
+        <v>2.629</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.05</v>
+        <v>10.5161</v>
       </c>
       <c r="R19" t="n">
-        <v>0.5</v>
+        <v>3.5327</v>
       </c>
       <c r="S19" t="n">
-        <v>0.1</v>
+        <v>4.688</v>
       </c>
       <c r="T19" t="n">
-        <v>0.1</v>
+        <v>13.1451</v>
       </c>
       <c r="U19" t="n">
-        <v>0.5</v>
+        <v>19.7176</v>
       </c>
       <c r="V19" t="n">
-        <v>0.05</v>
+        <v>2.649</v>
       </c>
     </row>
     <row r="20">
@@ -1676,61 +1653,61 @@
         <v>91</v>
       </c>
       <c r="D20" t="n">
-        <v>1000</v>
+        <v>400</v>
       </c>
       <c r="E20" t="n">
-        <v>1</v>
+        <v>23.953</v>
       </c>
       <c r="F20" t="n">
-        <v>0.1</v>
+        <v>17.06</v>
       </c>
       <c r="G20" t="n">
-        <v>1</v>
+        <v>23.7</v>
       </c>
       <c r="H20" t="n">
-        <v>10</v>
+        <v>18.96</v>
       </c>
       <c r="I20" t="n">
-        <v>1</v>
+        <v>279.85</v>
       </c>
       <c r="J20" t="n">
-        <v>0.5</v>
+        <v>243.87</v>
       </c>
       <c r="K20" t="n">
-        <v>0.1</v>
+        <v>83.95</v>
       </c>
       <c r="L20" t="n">
-        <v>0.1</v>
+        <v>5.597</v>
       </c>
       <c r="M20" t="n">
-        <v>0.5</v>
+        <v>293.84</v>
       </c>
       <c r="N20" t="n">
-        <v>0</v>
+        <v>2.808</v>
       </c>
       <c r="O20" t="n">
-        <v>0</v>
+        <v>140.675</v>
       </c>
       <c r="P20" t="n">
-        <v>0.1</v>
+        <v>2.8135</v>
       </c>
       <c r="Q20" t="n">
-        <v>0.05</v>
+        <v>11.254</v>
       </c>
       <c r="R20" t="n">
-        <v>0.5</v>
+        <v>4.0004</v>
       </c>
       <c r="S20" t="n">
-        <v>0.1</v>
+        <v>4.844</v>
       </c>
       <c r="T20" t="n">
-        <v>0.1</v>
+        <v>14.0675</v>
       </c>
       <c r="U20" t="n">
-        <v>0.5</v>
+        <v>21.1013</v>
       </c>
       <c r="V20" t="n">
-        <v>0.05</v>
+        <v>2.8335</v>
       </c>
     </row>
     <row r="21">
@@ -1744,61 +1721,61 @@
         <v>96</v>
       </c>
       <c r="D21" t="n">
-        <v>1000</v>
+        <v>400</v>
       </c>
       <c r="E21" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="F21" t="n">
-        <v>0.1</v>
+        <v>18</v>
       </c>
       <c r="G21" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="H21" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="I21" t="n">
-        <v>1</v>
+        <v>300</v>
       </c>
       <c r="J21" t="n">
-        <v>0.5</v>
+        <v>282.86</v>
       </c>
       <c r="K21" t="n">
-        <v>0.1</v>
+        <v>90</v>
       </c>
       <c r="L21" t="n">
-        <v>0.1</v>
+        <v>6</v>
       </c>
       <c r="M21" t="n">
-        <v>0.5</v>
+        <v>315</v>
       </c>
       <c r="N21" t="n">
-        <v>0</v>
+        <v>3.01</v>
       </c>
       <c r="O21" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="P21" t="n">
-        <v>0.1</v>
+        <v>3</v>
       </c>
       <c r="Q21" t="n">
-        <v>0.05</v>
+        <v>12</v>
       </c>
       <c r="R21" t="n">
-        <v>0.5</v>
+        <v>4.5</v>
       </c>
       <c r="S21" t="n">
-        <v>0.1</v>
+        <v>5</v>
       </c>
       <c r="T21" t="n">
-        <v>0.1</v>
+        <v>15</v>
       </c>
       <c r="U21" t="n">
-        <v>0.5</v>
+        <v>22.5</v>
       </c>
       <c r="V21" t="n">
-        <v>0.05</v>
+        <v>3.02</v>
       </c>
     </row>
   </sheetData>
@@ -1815,18 +1792,8 @@
   <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr"/>
-      <c r="B1" t="inlineStr"/>
-      <c r="C1" t="inlineStr"/>
-      <c r="D1" t="inlineStr"/>
-      <c r="E1" t="inlineStr"/>
-    </row>
+    <row r="1"/>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
         <v>1</v>
       </c>

</xml_diff>